<commit_message>
Update V106A susc; update binding energies and plots
</commit_message>
<xml_diff>
--- a/manuscript/Supplementary-Table-1.xlsx
+++ b/manuscript/Supplementary-Table-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rohitpro/Career/00_Github/nnrti-mechanisms/manuscript/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{857580D9-CA0B-C140-9684-45CA0E4187C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E395AB-F59E-F64D-8CC0-A3CB5087AFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="66960" yWindow="-5900" windowWidth="35880" windowHeight="15940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="15960" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="192">
   <si>
     <t>V106A</t>
   </si>
@@ -127,12 +127,6 @@
     <t>[1.2, 1.3, 1.5, 6.0]</t>
   </si>
   <si>
-    <t>[0.4, 11, 20]</t>
-  </si>
-  <si>
-    <t>[7.1, 28]</t>
-  </si>
-  <si>
     <t>Primary Source Studies (URLs)</t>
   </si>
   <si>
@@ -608,6 +602,18 @@
   </si>
   <si>
     <t>[36]</t>
+  </si>
+  <si>
+    <t>[https://pubmed.ncbi.nlm.nih.gov/34570651/]</t>
+  </si>
+  <si>
+    <t>Unavailable (see Table 2 in source study)</t>
+  </si>
+  <si>
+    <t>[7.1, 9.6, 28]</t>
+  </si>
+  <si>
+    <t>[https://pubmed.ncbi.nlm.nih.gov/24379202/, https://pubmed.ncbi.nlm.nih.gov/25385110/]</t>
   </si>
 </sst>
 </file>
@@ -647,11 +653,11 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1254,6 +1260,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E498A9B6-C31F-3269-08A7-6438721E9B93}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9093200" y="1079500"/>
+          <a:ext cx="6629400" cy="5511800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1656,9 +1706,9 @@
   <cols>
     <col min="1" max="1" width="19.6640625" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="28.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="149.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="56.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="82.6640625" bestFit="1" customWidth="1"/>
@@ -1667,27 +1717,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>31</v>
+      <c r="F1" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B2" t="s">
@@ -1703,11 +1753,11 @@
         <v>26</v>
       </c>
       <c r="F2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="1"/>
+      <c r="A3" s="3"/>
       <c r="B3" t="s">
         <v>13</v>
       </c>
@@ -1718,14 +1768,14 @@
         <v>6</v>
       </c>
       <c r="E3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="1"/>
+      <c r="A4" s="3"/>
       <c r="B4" t="s">
         <v>2</v>
       </c>
@@ -1739,11 +1789,11 @@
         <v>28</v>
       </c>
       <c r="F4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="1"/>
+      <c r="A5" s="3"/>
       <c r="B5" t="s">
         <v>14</v>
       </c>
@@ -1757,11 +1807,11 @@
         <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B6" t="s">
@@ -1774,32 +1824,32 @@
         <v>3</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>189</v>
       </c>
       <c r="F6" t="s">
-        <v>122</v>
+        <v>188</v>
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="1"/>
+      <c r="A7" s="3"/>
       <c r="B7" t="s">
         <v>0</v>
       </c>
       <c r="C7">
-        <v>18</v>
+        <v>9.6</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>30</v>
+        <v>190</v>
       </c>
       <c r="F7" t="s">
-        <v>71</v>
+        <v>191</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="1"/>
+      <c r="A8" s="3"/>
       <c r="B8" t="s">
         <v>16</v>
       </c>
@@ -1810,14 +1860,14 @@
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="1"/>
+      <c r="A9" s="3"/>
       <c r="B9" t="s">
         <v>11</v>
       </c>
@@ -1828,14 +1878,14 @@
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="1"/>
+      <c r="A10" s="3"/>
       <c r="B10" t="s">
         <v>10</v>
       </c>
@@ -1846,14 +1896,14 @@
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F10" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="1"/>
+      <c r="A11" s="3"/>
       <c r="B11" t="s">
         <v>3</v>
       </c>
@@ -1864,14 +1914,14 @@
         <v>6</v>
       </c>
       <c r="E11" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F11" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="1"/>
+      <c r="A12" s="3"/>
       <c r="B12" t="s">
         <v>9</v>
       </c>
@@ -1882,14 +1932,14 @@
         <v>2</v>
       </c>
       <c r="E12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F12" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="1"/>
+      <c r="A13" s="3"/>
       <c r="B13" t="s">
         <v>12</v>
       </c>
@@ -1900,14 +1950,14 @@
         <v>2</v>
       </c>
       <c r="E13" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F13" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B14" t="s">
@@ -1920,14 +1970,14 @@
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="1"/>
+      <c r="A15" s="3"/>
       <c r="B15" t="s">
         <v>5</v>
       </c>
@@ -1938,14 +1988,14 @@
         <v>4</v>
       </c>
       <c r="E15" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="1"/>
+      <c r="A16" s="3"/>
       <c r="B16" t="s">
         <v>23</v>
       </c>
@@ -1956,14 +2006,14 @@
         <v>8</v>
       </c>
       <c r="E16" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="1"/>
+      <c r="A17" s="3"/>
       <c r="B17" t="s">
         <v>7</v>
       </c>
@@ -1974,14 +2024,14 @@
         <v>2</v>
       </c>
       <c r="E17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="1"/>
+      <c r="A18" s="3"/>
       <c r="B18" t="s">
         <v>4</v>
       </c>
@@ -1992,14 +2042,14 @@
         <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="1"/>
+      <c r="A19" s="3"/>
       <c r="B19" t="s">
         <v>8</v>
       </c>
@@ -2010,10 +2060,10 @@
         <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F19" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -2039,77 +2089,77 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I2" s="3">
+        <v>43</v>
+      </c>
+      <c r="I2" s="2">
         <v>2000</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>150</v>
@@ -2117,22 +2167,22 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>106</v>
@@ -2140,25 +2190,25 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5">
         <v>100</v>
@@ -2177,54 +2227,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E2" t="s">
         <v>3</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>95</v>
@@ -2232,16 +2282,16 @@
     </row>
     <row r="3" spans="1:10">
       <c r="C3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E3" t="s">
         <v>3</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>116</v>
@@ -2249,16 +2299,16 @@
     </row>
     <row r="4" spans="1:10">
       <c r="C4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E4" t="s">
         <v>3</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>116</v>
@@ -2266,10 +2316,10 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
         <v>3</v>
@@ -2278,10 +2328,10 @@
         <v>3</v>
       </c>
       <c r="G5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5">
         <v>31</v>
@@ -2289,10 +2339,10 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s">
         <v>3</v>
@@ -2301,10 +2351,10 @@
         <v>3</v>
       </c>
       <c r="G6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I6">
         <v>158</v>
@@ -2312,25 +2362,25 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
         <v>3</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I7">
         <v>181</v>
@@ -2338,25 +2388,25 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E8" t="s">
         <v>3</v>
       </c>
       <c r="G8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I8">
         <v>181</v>
@@ -2373,10 +2423,10 @@
         <v>3</v>
       </c>
       <c r="G9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I9">
         <v>100</v>
@@ -2387,22 +2437,22 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C10" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E10" t="s">
         <v>3</v>
       </c>
       <c r="G10" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I10">
         <v>89</v>
@@ -2410,25 +2460,25 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D11" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E11" t="s">
         <v>3</v>
       </c>
       <c r="G11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H11" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I11">
         <v>182</v>
@@ -2436,25 +2486,25 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E12" t="s">
         <v>3</v>
       </c>
       <c r="G12" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I12">
         <v>100</v>
@@ -2473,57 +2523,57 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>210</v>
@@ -2534,28 +2584,28 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>95</v>
@@ -2574,54 +2624,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="G2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>173</v>
@@ -2629,22 +2679,22 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C3" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="G3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>150</v>
@@ -2663,54 +2713,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E2" t="s">
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>3.4</v>
@@ -2718,22 +2768,22 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C3" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E3" t="s">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>17</v>
@@ -2752,54 +2802,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E2" t="s">
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>1.5</v>
@@ -2807,16 +2857,16 @@
     </row>
     <row r="3" spans="1:10">
       <c r="C3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E3" t="s">
         <v>5</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>4.5</v>
@@ -2824,16 +2874,16 @@
     </row>
     <row r="4" spans="1:10">
       <c r="C4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E4" t="s">
         <v>5</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>5.9</v>
@@ -2841,16 +2891,16 @@
     </row>
     <row r="5" spans="1:10">
       <c r="C5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E5" t="s">
         <v>5</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5">
         <v>11</v>
@@ -2858,10 +2908,10 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -2870,10 +2920,10 @@
         <v>5</v>
       </c>
       <c r="G6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I6">
         <v>6.6</v>
@@ -2892,54 +2942,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>2.7</v>
@@ -2947,16 +2997,16 @@
     </row>
     <row r="3" spans="1:10">
       <c r="C3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E3" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>4.5</v>
@@ -2964,16 +3014,16 @@
     </row>
     <row r="4" spans="1:10">
       <c r="C4" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>4.5999999999999996</v>
@@ -2981,16 +3031,16 @@
     </row>
     <row r="5" spans="1:10">
       <c r="C5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5">
         <v>5.0999999999999996</v>
@@ -2998,16 +3048,16 @@
     </row>
     <row r="6" spans="1:10">
       <c r="C6" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I6">
         <v>8.4</v>
@@ -3015,16 +3065,16 @@
     </row>
     <row r="7" spans="1:10">
       <c r="C7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E7" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I7">
         <v>10</v>
@@ -3032,16 +3082,16 @@
     </row>
     <row r="8" spans="1:10">
       <c r="C8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I8">
         <v>11</v>
@@ -3049,16 +3099,16 @@
     </row>
     <row r="9" spans="1:10">
       <c r="C9" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E9" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I9">
         <v>19</v>
@@ -3066,22 +3116,22 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" t="s">
+        <v>176</v>
+      </c>
+      <c r="E10" t="s">
+        <v>175</v>
+      </c>
+      <c r="G10" t="s">
         <v>58</v>
       </c>
-      <c r="B10" t="s">
-        <v>59</v>
-      </c>
-      <c r="C10" t="s">
-        <v>178</v>
-      </c>
-      <c r="E10" t="s">
-        <v>177</v>
-      </c>
-      <c r="G10" t="s">
-        <v>60</v>
-      </c>
       <c r="H10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I10">
         <v>5.7</v>
@@ -3089,22 +3139,22 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E11" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H11" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I11">
         <v>3</v>
@@ -3112,22 +3162,22 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G12" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I12">
         <v>6.3</v>
@@ -3146,54 +3196,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>5.7</v>
@@ -3201,16 +3251,16 @@
     </row>
     <row r="3" spans="1:10">
       <c r="C3" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E3" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>10</v>
@@ -3218,22 +3268,22 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>38</v>
@@ -3241,22 +3291,22 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E5" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5">
         <v>9.6999999999999993</v>
@@ -3275,54 +3325,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E2" t="s">
         <v>4</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>18</v>
@@ -3341,54 +3391,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>36</v>
@@ -3416,54 +3466,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E2" t="s">
         <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>1.4</v>
@@ -3471,28 +3521,28 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" t="s">
         <v>46</v>
-      </c>
-      <c r="B3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D3" t="s">
-        <v>48</v>
       </c>
       <c r="E3" t="s">
         <v>15</v>
       </c>
       <c r="F3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>1</v>
@@ -3500,22 +3550,22 @@
     </row>
     <row r="4" spans="1:10">
       <c r="C4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E4" t="s">
         <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>1.8</v>
@@ -3523,22 +3573,22 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" t="s">
         <v>53</v>
-      </c>
-      <c r="B5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C5" t="s">
-        <v>55</v>
       </c>
       <c r="E5" t="s">
         <v>15</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5">
         <v>0.8</v>
@@ -3557,54 +3607,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E2" t="s">
         <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>0.6</v>
@@ -3612,16 +3662,16 @@
     </row>
     <row r="3" spans="1:10">
       <c r="C3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E3" t="s">
         <v>13</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>1.2</v>
@@ -3629,16 +3679,16 @@
     </row>
     <row r="4" spans="1:10">
       <c r="C4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E4" t="s">
         <v>13</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>1.2</v>
@@ -3646,16 +3696,16 @@
     </row>
     <row r="5" spans="1:10">
       <c r="C5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E5" t="s">
         <v>13</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5">
         <v>1.3</v>
@@ -3663,16 +3713,16 @@
     </row>
     <row r="6" spans="1:10">
       <c r="C6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E6" t="s">
         <v>13</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I6">
         <v>3</v>
@@ -3680,19 +3730,19 @@
     </row>
     <row r="7" spans="1:10">
       <c r="C7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E7" t="s">
         <v>13</v>
       </c>
       <c r="F7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I7">
         <v>2.8</v>
@@ -3700,10 +3750,10 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C8" t="s">
         <v>13</v>
@@ -3712,10 +3762,10 @@
         <v>13</v>
       </c>
       <c r="G8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I8">
         <v>1.8</v>
@@ -3723,10 +3773,10 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C9" t="s">
         <v>13</v>
@@ -3735,10 +3785,10 @@
         <v>13</v>
       </c>
       <c r="G9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I9">
         <v>7</v>
@@ -3746,25 +3796,25 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E10" t="s">
         <v>13</v>
       </c>
       <c r="G10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I10">
         <v>0.4</v>
@@ -3772,22 +3822,22 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" t="s">
         <v>66</v>
-      </c>
-      <c r="B11" t="s">
-        <v>59</v>
-      </c>
-      <c r="C11" t="s">
-        <v>68</v>
       </c>
       <c r="E11" t="s">
         <v>13</v>
       </c>
       <c r="G11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H11" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I11">
         <v>1</v>
@@ -3806,54 +3856,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E2" t="s">
         <v>2</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>1.2</v>
@@ -3861,16 +3911,16 @@
     </row>
     <row r="3" spans="1:10">
       <c r="C3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E3" t="s">
         <v>2</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>1.3</v>
@@ -3878,16 +3928,16 @@
     </row>
     <row r="4" spans="1:10">
       <c r="C4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E4" t="s">
         <v>2</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>1.5</v>
@@ -3895,16 +3945,16 @@
     </row>
     <row r="5" spans="1:10">
       <c r="C5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E5" t="s">
         <v>2</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5">
         <v>6</v>
@@ -3912,10 +3962,10 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s">
         <v>2</v>
@@ -3924,10 +3974,10 @@
         <v>2</v>
       </c>
       <c r="G6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I6">
         <v>2.8</v>
@@ -3935,10 +3985,10 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C7" t="s">
         <v>2</v>
@@ -3947,10 +3997,10 @@
         <v>2</v>
       </c>
       <c r="G7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I7">
         <v>3.1</v>
@@ -3958,28 +4008,28 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E8" t="s">
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I8">
         <v>1.4</v>
@@ -3987,22 +4037,22 @@
     </row>
     <row r="9" spans="1:10">
       <c r="C9" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E9" t="s">
         <v>2</v>
       </c>
       <c r="F9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I9">
         <v>0.6</v>
@@ -4010,22 +4060,22 @@
     </row>
     <row r="10" spans="1:10">
       <c r="C10" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E10" t="s">
         <v>2</v>
       </c>
       <c r="F10" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I10">
         <v>0.8</v>
@@ -4033,22 +4083,22 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E11" t="s">
         <v>2</v>
       </c>
       <c r="G11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H11" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I11">
         <v>0.4</v>
@@ -4056,25 +4106,25 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D12" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E12" t="s">
         <v>2</v>
       </c>
       <c r="G12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I12">
         <v>2.6</v>
@@ -4093,54 +4143,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E2" t="s">
         <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>1.8</v>
@@ -4148,16 +4198,16 @@
     </row>
     <row r="3" spans="1:10">
       <c r="C3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E3" t="s">
         <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>3.6</v>
@@ -4165,10 +4215,10 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C4" t="s">
         <v>14</v>
@@ -4177,10 +4227,10 @@
         <v>14</v>
       </c>
       <c r="G4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>5.5</v>
@@ -4188,10 +4238,10 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
         <v>14</v>
@@ -4200,10 +4250,10 @@
         <v>14</v>
       </c>
       <c r="G5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5">
         <v>1.8</v>
@@ -4211,22 +4261,22 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E6" t="s">
         <v>14</v>
       </c>
       <c r="G6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I6">
         <v>2.5</v>
@@ -4244,57 +4294,57 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" t="s">
         <v>84</v>
       </c>
-      <c r="B2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>85</v>
       </c>
-      <c r="D2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E2" t="s">
-        <v>87</v>
-      </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>210</v>
@@ -4302,22 +4352,22 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>44</v>
@@ -4328,22 +4378,22 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G4" t="s">
         <v>90</v>
       </c>
-      <c r="B4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E4" t="s">
-        <v>91</v>
-      </c>
-      <c r="G4" t="s">
-        <v>92</v>
-      </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>226</v>
@@ -4351,33 +4401,33 @@
     </row>
     <row r="5" spans="1:10">
       <c r="C5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="G5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
-      </c>
-      <c r="I5" s="3">
+        <v>43</v>
+      </c>
+      <c r="I5" s="2">
         <v>1558</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="C6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I6">
         <v>854</v>
@@ -4385,36 +4435,36 @@
     </row>
     <row r="7" spans="1:10">
       <c r="C7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E7" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H7" t="s">
-        <v>45</v>
-      </c>
-      <c r="I7" s="3">
+        <v>43</v>
+      </c>
+      <c r="I7" s="2">
         <v>10000</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="C8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E8" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I8">
         <v>68</v>
@@ -4422,33 +4472,33 @@
     </row>
     <row r="9" spans="1:10">
       <c r="C9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
-      </c>
-      <c r="I9" s="3">
+        <v>43</v>
+      </c>
+      <c r="I9" s="2">
         <v>4167</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="C10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I10">
         <v>850</v>
@@ -4456,42 +4506,42 @@
     </row>
     <row r="11" spans="1:10">
       <c r="C11" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E11" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H11" t="s">
-        <v>45</v>
-      </c>
-      <c r="I11" s="3">
+        <v>43</v>
+      </c>
+      <c r="I11" s="2">
         <v>50000</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
+        <v>98</v>
+      </c>
+      <c r="B12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" t="s">
+        <v>115</v>
+      </c>
+      <c r="D12" t="s">
+        <v>99</v>
+      </c>
+      <c r="E12" t="s">
         <v>100</v>
       </c>
-      <c r="B12" t="s">
-        <v>59</v>
-      </c>
-      <c r="C12" t="s">
-        <v>117</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="G12" t="s">
         <v>101</v>
       </c>
-      <c r="E12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G12" t="s">
-        <v>103</v>
-      </c>
       <c r="H12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I12">
         <v>537</v>
@@ -4499,25 +4549,25 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E13" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H13" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I13">
         <v>11</v>
@@ -4525,19 +4575,19 @@
     </row>
     <row r="14" spans="1:10">
       <c r="C14" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G14" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H14" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I14">
         <v>211</v>
@@ -4545,19 +4595,19 @@
     </row>
     <row r="15" spans="1:10">
       <c r="C15" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E15" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H15" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I15">
         <v>0.4</v>
@@ -4565,16 +4615,16 @@
     </row>
     <row r="16" spans="1:10">
       <c r="C16" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E16" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G16" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I16">
         <v>20</v>
@@ -4593,54 +4643,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E2" t="s">
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>7.1</v>
@@ -4648,16 +4698,16 @@
     </row>
     <row r="3" spans="1:10">
       <c r="C3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E3" t="s">
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>28</v>
@@ -4665,10 +4715,10 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C4" t="s">
         <v>0</v>
@@ -4677,10 +4727,10 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>9.6</v>
@@ -4688,10 +4738,10 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
         <v>0</v>
@@ -4700,10 +4750,10 @@
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5">
         <v>23</v>
@@ -4711,22 +4761,22 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E6" t="s">
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I6">
         <v>13</v>
@@ -4734,25 +4784,25 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I7">
         <v>2.2999999999999998</v>
@@ -4771,57 +4821,57 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>93</v>
@@ -4829,25 +4879,25 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>93</v>
@@ -4858,16 +4908,16 @@
     </row>
     <row r="4" spans="1:10">
       <c r="C4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>100</v>
@@ -4878,25 +4928,25 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5">
         <v>97</v>
@@ -4915,54 +4965,54 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <v>105</v>
@@ -4970,22 +5020,22 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I3">
         <v>105</v>
@@ -4996,16 +5046,16 @@
     </row>
     <row r="4" spans="1:10">
       <c r="C4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4">
         <v>100</v>
@@ -5016,25 +5066,25 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5">
         <v>66</v>
@@ -5042,25 +5092,25 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I6">
         <v>102</v>

</xml_diff>